<commit_message>
Improve URL generator run failures
</commit_message>
<xml_diff>
--- a/public/templates/url-generator-orders-template.xlsx
+++ b/public/templates/url-generator-orders-template.xlsx
@@ -28,7 +28,7 @@
     <t>ABC-123</t>
   </si>
   <si>
-    <t>https://example.com/product</t>
+    <t>https://example.com</t>
   </si>
 </sst>
 </file>
@@ -449,6 +449,6 @@
   </sheetData>
   <autoFilter ref="A1:C2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>